<commit_message>
I linked the movement system questions to the quiz system in a way that was suitable for the data structure. And i made changes to the dataset.
</commit_message>
<xml_diff>
--- a/ai/data/raw/Project_MovementSystem_QDatas.xlsx
+++ b/ai/data/raw/Project_MovementSystem_QDatas.xlsx
@@ -85,7 +85,7 @@
     <t>Os Frontale, doğumda 2 parça halinde olup 1–2 yaşlarında kemikleşerek tek parça hâline dönüşür.</t>
   </si>
   <si>
-    <t>{"options":["True","False"]}</t>
+    <t>{"options":["Doğru","Yanlış"]}</t>
   </si>
   <si>
     <t>{"correct_index":1}</t>
@@ -764,11 +764,7 @@
     <t>Göğüs tahtası kemiğini oluşturan 3 kısmın üstten alta doğru isimleri nelerdir?</t>
   </si>
   <si>
-    <t>{"options":["hançersi çıkıntı/sternum
-gövdesi/sternum sapı","sternum sapı/sternum
-gövdesi/hançersi çıkıntı","sternum
-gövdesi/hançersi çıkıntı/sternum sapı","sternum
-gövdesi/sternum sapı/hançersi çıkıntı"]}</t>
+    <t>{"options":["hançersi çıkıntı/sternum gövdesi/sternum sapı","sternum sapı/sternum gövdesi/hançersi çıkıntı","sternum gövdesi/hançersi çıkıntı/sternum sapı","sternum gövdesi/sternum sapı/hançersi çıkıntı"]}</t>
   </si>
   <si>
     <t>Sternumun bölümlerini yukarıdan aşağıya sıralarken sap, gövde ve uç kısmı düşün.</t>
@@ -927,8 +923,7 @@
     <t>antebrachium; ön kol; döner kemik; avuç içi</t>
   </si>
   <si>
-    <t>Öne uzatılan elin avuç içi aşağı çevrildiğinde os radius, ulnanın üzerine
-doğru döner.</t>
+    <t>Öne uzatılan elin avuç içi aşağı çevrildiğinde os radius, ulnanın üzerine doğru döner.</t>
   </si>
   <si>
     <t>Pronasyon sırasında radiusun ulna ile ilişkisini gözünde canlandır.</t>
@@ -1202,8 +1197,7 @@
     <t>Tibia'nın üst kısmı hangi kemik ile eklem yapar?</t>
   </si>
   <si>
-    <t xml:space="preserve">{"options":["Patella","Fibula","Femur","Talus"]}
-</t>
+    <t>{"options":["Patella","Fibula","Femur","Talus"]}</t>
   </si>
   <si>
     <t>Tibianın üstte diz eklemine hangi kemikle katıldığını hatırla.</t>
@@ -1224,8 +1218,7 @@
     <t>Tek ayakta kaç adet ossa metatarsi bulunur?</t>
   </si>
   <si>
-    <t xml:space="preserve">{"options":["5","7","10","14"]}
-</t>
+    <t>{"options":["5","7","10","14"]}</t>
   </si>
   <si>
     <t xml:space="preserve">{"correct_index":0}
@@ -1484,7 +1477,7 @@
     <t>Burkulmada ayrılma geçicidir, kalıcı ayrılma ise çıkıktır.</t>
   </si>
   <si>
-    <t>ers kitabına göre, burkulma eklemi oluşturan kemiklerin ani olarak anatomik pozisyonlarını kaybederek eklem yüzlerinin geçici olarak ayrılmasıdır; kalıcı değildir</t>
+    <t>Ders kitabına göre, burkulma eklemi oluşturan kemiklerin ani olarak anatomik pozisyonlarını kaybederek eklem yüzlerinin geçici olarak ayrılmasıdır; kalıcı değildir</t>
   </si>
   <si>
     <t>fibrous_joint_mcq_01</t>
@@ -1804,7 +1797,7 @@
 4. M. Masseter</t>
   </si>
   <si>
-    <t>{"options":["Çiğneme-Mimik-Çiğneme-Mimik", "Mimik-Çiğneme-Mimik-Çiğneme", "Çiğneme-Mimik-Mimik-Çiğneme", "Mimik-Çiğneme-Çiğneme-Mimik"]}</t>
+    <t>{"options":["Çiğneme-Mimik-Çiğneme-Mimik", "Mimik-Çiğneme-Mimik-Çiğneme", "Çiğneme-Mimik-Mimik Çiğneme", "Mimik-Çiğneme-Çiğneme Mimik"]}</t>
   </si>
   <si>
     <t>M. temporalis ve M. masseter çiğneme; orbicularis oris ve risorius mimik kasıdır.</t>
@@ -1822,8 +1815,7 @@
     <t>kas; boyun; fleksiyon; kalın; yüzeysel</t>
   </si>
   <si>
-    <t>M. Sternocleidomastoideus, tek taraflı kasılınca başı kendi tarafına eğer, yüzü
-karşı tarafa baktırır. Çift taraflı kasılırsa başa fleksiyon yaptırır.</t>
+    <t>M. Sternocleidomastoideus, tek taraflı kasılınca başı kendi tarafına eğer, yüzü karşı tarafa baktırır. Çift taraflı kasılırsa başa fleksiyon yaptırır.</t>
   </si>
   <si>
     <t>SCM’nin tek taraflı ve çift taraflı kasılmalarındaki etkileri ayrı ayrı düşün.</t>
@@ -2058,8 +2050,7 @@
     <t>Baldırın arka kısmında bulunan ve topuk kemiğine Aşil tendonu ile bağlanan kas grubunu düşün.</t>
   </si>
   <si>
-    <t>Ders kitabına göre, M. Triceps Surae iki kas tibianın üst ucundan başlayıp aşil tendonunu oluşturduktan sonra topuk
-kemiğinde sonlanır.</t>
+    <t>Ders kitabına göre, M. Triceps Surae iki kas tibianın üst ucundan başlayıp aşil tendonunu oluşturduktan sonra topuk kemiğinde sonlanır.</t>
   </si>
   <si>
     <t>Ders kitabı s.83</t>
@@ -4542,7 +4533,7 @@
       <c r="J49" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="K49" s="2" t="s">
+      <c r="K49" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L49" s="2" t="s">
@@ -4587,7 +4578,7 @@
       <c r="J50" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="K50" s="2" t="s">
+      <c r="K50" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L50" s="2" t="s">
@@ -4632,7 +4623,7 @@
       <c r="J51" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="K51" s="2" t="s">
+      <c r="K51" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L51" s="2" t="s">
@@ -4679,7 +4670,7 @@
       <c r="J52" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="K52" s="2" t="s">
+      <c r="K52" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L52" s="2" t="s">
@@ -4724,7 +4715,7 @@
       <c r="J53" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="K53" s="2" t="s">
+      <c r="K53" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L53" s="2" t="s">
@@ -4771,7 +4762,7 @@
       <c r="J54" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="K54" s="2" t="s">
+      <c r="K54" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L54" s="2" t="s">
@@ -4818,7 +4809,7 @@
       <c r="J55" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="K55" s="2" t="s">
+      <c r="K55" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L55" s="4" t="s">
@@ -4863,7 +4854,7 @@
       <c r="J56" s="2" t="s">
         <v>364</v>
       </c>
-      <c r="K56" s="2" t="s">
+      <c r="K56" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L56" s="2" t="s">
@@ -4908,7 +4899,7 @@
       <c r="J57" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="K57" s="2" t="s">
+      <c r="K57" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L57" s="2" t="s">
@@ -4953,7 +4944,7 @@
       <c r="J58" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="K58" s="2" t="s">
+      <c r="K58" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L58" s="2" t="s">
@@ -5063,7 +5054,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="2" t="s">
         <v>390</v>
       </c>
@@ -5094,7 +5085,7 @@
       <c r="J61" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="K61" s="2" t="s">
+      <c r="K61" s="4" t="s">
         <v>394</v>
       </c>
       <c r="L61" s="2" t="s">
@@ -5141,7 +5132,7 @@
       <c r="J62" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="K62" s="2" t="s">
+      <c r="K62" s="4" t="s">
         <v>401</v>
       </c>
       <c r="L62" s="2" t="s">
@@ -5329,7 +5320,7 @@
       <c r="J66" s="2" t="s">
         <v>428</v>
       </c>
-      <c r="K66" s="2" t="s">
+      <c r="K66" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L66" s="2" t="s">
@@ -5376,7 +5367,7 @@
       <c r="J67" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="K67" s="2" t="s">
+      <c r="K67" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L67" s="2" t="s">
@@ -5421,7 +5412,7 @@
       <c r="J68" s="2" t="s">
         <v>441</v>
       </c>
-      <c r="K68" s="2" t="s">
+      <c r="K68" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L68" s="2" t="s">
@@ -5468,7 +5459,7 @@
       <c r="J69" s="2" t="s">
         <v>448</v>
       </c>
-      <c r="K69" s="2" t="s">
+      <c r="K69" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L69" s="2" t="s">
@@ -5515,7 +5506,7 @@
       <c r="J70" s="2" t="s">
         <v>455</v>
       </c>
-      <c r="K70" s="2" t="s">
+      <c r="K70" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L70" s="2" t="s">
@@ -5562,7 +5553,7 @@
       <c r="J71" s="2" t="s">
         <v>462</v>
       </c>
-      <c r="K71" s="2" t="s">
+      <c r="K71" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L71" s="2" t="s">
@@ -5607,7 +5598,7 @@
       <c r="J72" s="2" t="s">
         <v>467</v>
       </c>
-      <c r="K72" s="2" t="s">
+      <c r="K72" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L72" s="2" t="s">
@@ -5654,7 +5645,7 @@
       <c r="J73" s="2" t="s">
         <v>473</v>
       </c>
-      <c r="K73" s="2" t="s">
+      <c r="K73" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L73" s="2" t="s">
@@ -5701,7 +5692,7 @@
       <c r="J74" s="2" t="s">
         <v>479</v>
       </c>
-      <c r="K74" s="2" t="s">
+      <c r="K74" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L74" s="2" t="s">
@@ -5748,7 +5739,7 @@
       <c r="J75" s="2" t="s">
         <v>485</v>
       </c>
-      <c r="K75" s="2" t="s">
+      <c r="K75" s="1" t="s">
         <v>24</v>
       </c>
       <c r="L75" s="2" t="s">
@@ -5757,7 +5748,7 @@
       <c r="M75" s="1" t="s">
         <v>486</v>
       </c>
-      <c r="N75" s="2" t="s">
+      <c r="N75" s="4" t="s">
         <v>487</v>
       </c>
       <c r="O75" s="2" t="s">

</xml_diff>

<commit_message>
I made changes to both the dataset and the scripts in order to integrate the match questions.
</commit_message>
<xml_diff>
--- a/ai/data/raw/Project_MovementSystem_QDatas.xlsx
+++ b/ai/data/raw/Project_MovementSystem_QDatas.xlsx
@@ -556,7 +556,7 @@
     <t>{"left":["Vertebrae cervicales", "Vertebrae lumbales", "Vertebrae sacrale", "Vertebrae thoracicae", "Vertebrae coccygea"], "right":["T1-T12", "L1-L5", "C1-C7", "Co1-Co4", "S1-S5"], "shuffle_right":true}</t>
   </si>
   <si>
-    <t>{"pairs":[[0,2], [1,1], [2,4], [3,0], [4,3]]}</t>
+    <t>{"pairs":[{"leftIndex":0,"rightIndex":2},{"leftIndex":1,"rightIndex":1},{"leftIndex":2,"rightIndex":4},{"leftIndex":3,"rightIndex":0},{"leftIndex":4,"rightIndex":3}]}</t>
   </si>
   <si>
     <t>Ders kitabı s.59</t>
@@ -857,7 +857,7 @@
     <t>{"left":["Köprücük kemiği ile eklem yapan dış yana doğru uzanan çıkıntı", "Üst dış yanda öne doğru uzanan ve bazı kasların tutunduğu gagaya benzer çıkıntı", "Kol kemiğiyle eklem yapan üst dış kenarı"], "right":["cavitas glenoidalis", "acromion", "processus coracoideus"], "shuffle_right":true}</t>
   </si>
   <si>
-    <t>{"pairs":[[0,1], [1,2], [2,0]]}</t>
+    <t>{"pairs":[{"leftIndex":0,"rightIndex":1},{"leftIndex":1,"rightIndex":2},{"leftIndex":2,"rightIndex":0}]}</t>
   </si>
   <si>
     <t>os_humerus_tf_01</t>
@@ -893,7 +893,7 @@
     <t>{"left":["trochlea humeri", "caput humeri", "capitulum humeri"], "right":["Kürek kemiği ile eklem (omuz eklemi) yapar.", "İç yandaki dirsek kemiği ile eklem yapar.", "Dış yandaki döner kemikle eklem yapar."], "shuffle_right":true}</t>
   </si>
   <si>
-    <t>{"pairs":[[0,1], [1,0], [2,2]]}</t>
+    <t>{"pairs":[{"leftIndex":0,"rightIndex":1},{"leftIndex":1,"rightIndex":0},{"leftIndex":2,"rightIndex":2}]}</t>
   </si>
   <si>
     <t>os_ulna_tf_01</t>
@@ -959,7 +959,7 @@
     <t>{"left":["Ossa Carpi", "Ossa Metacarpi", "Ossa Digitorum Manus (Phalanges)"], "right":["4’erli iki sıra halinde 8 kısa kemik bulunur.", "Avuç içi ve el sırtının iskeletini oluşturan 5 uzun kemiktir.", "Beş parmakta toplam 14 kemik bulunur."], "shuffle_right":true}</t>
   </si>
   <si>
-    <t>{"pairs":[[0,0], [1,1], [2,2]]}</t>
+    <t>{"pairs":[{"leftIndex":0,"rightIndex":0},{"leftIndex":1,"rightIndex":1},{"leftIndex":2,"rightIndex":2}]}</t>
   </si>
   <si>
     <t>Ders kitabı s.63</t>
@@ -1757,7 +1757,7 @@
     <t>{"left":["quadriceps", "trapezoid", "latissimus" , "supinator"], "right":["Gövde şekline göre", "Yaptıkları işleve göre", "Baş sayısına göre" , "Büyüklüklerine göre"], "shuffle_right":true}</t>
   </si>
   <si>
-    <t>{"pairs":[[0,2], [1,0], [2,3], [3,1]]}</t>
+    <t>{"pairs":[{"leftIndex":0,"rightIndex":2},{"leftIndex":1,"rightIndex":0},{"leftIndex":2,"rightIndex":3},{"leftIndex":3,"rightIndex":1}]}</t>
   </si>
   <si>
     <t>muscle_matching_01</t>
@@ -1775,7 +1775,7 @@
     <t>{"left":["Tendon", "Fascia", "Bursa synovialis" , "Vagina synovialis tendinis"], "right":["Kasların hem tek tek hem de toplu halde kasılmasına yardım eder.", "Kasların kemiklere tutunmasını sağlayan yapıdır.", "Kemik veya diğer sert kısımlardan geçen tendonları bir kılıf gibi saran, içinde sinovyal sıvı bulunan kesedir." , "Çıkıntılı kemik kısımlar ile kas ve tendon arasına koruyucu bir yastık gibi giren, içinde sinovyal sıvı bulunan kesedir."], "shuffle_right":true}</t>
   </si>
   <si>
-    <t>{"pairs":[[0,1], [1,0], [2,3], [3,2]]}</t>
+    <t>{"pairs":[{"leftIndex":0,"rightIndex":1},{"leftIndex":1,"rightIndex":0},{"leftIndex":2,"rightIndex":3},{"leftIndex":3,"rightIndex":2}]}</t>
   </si>
   <si>
     <t>Ders kitabı s.75</t>
@@ -2325,6 +2325,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="24.13"/>
+    <col customWidth="1" min="12" max="12" width="14.63"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>